<commit_message>
Modif de la liste de composants
</commit_message>
<xml_diff>
--- a/lib/Liste des composants.xlsx
+++ b/lib/Liste des composants.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\loube\Desktop\Lib data\lib\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D27D136-A841-444D-8406-92A14259FC28}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC992A5D-9C35-41BC-9338-FD36A7C85B91}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="454" uniqueCount="157">
   <si>
     <t>nom du composant</t>
   </si>
@@ -445,9 +445,6 @@
     <t>Bouton</t>
   </si>
   <si>
-    <t>SWITCH TACTILE SPST 400gf SMD</t>
-  </si>
-  <si>
     <t>SMD-4P,4.2x3.2mm</t>
   </si>
   <si>
@@ -491,6 +488,9 @@
   </si>
   <si>
     <t>Generic connector, single row, 01x04 1.5mm</t>
+  </si>
+  <si>
+    <t>SWITCH TACTILE SPST 400gf SMD Push button switch,</t>
   </si>
 </sst>
 </file>
@@ -693,22 +693,6 @@
   </cellStyles>
   <dxfs count="4">
     <dxf>
-      <border>
-        <left style="thin">
-          <color rgb="FF356854"/>
-        </left>
-        <right style="thin">
-          <color rgb="FF356854"/>
-        </right>
-        <top style="thin">
-          <color rgb="FF356854"/>
-        </top>
-        <bottom style="thin">
-          <color rgb="FF356854"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFF6F8F9"/>
@@ -732,13 +716,29 @@
         </patternFill>
       </fill>
     </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="1" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16">
     <tableStyle name="Feuille 1-style" pivot="0" count="4" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
-      <tableStyleElement type="wholeTable" size="0" dxfId="0"/>
-      <tableStyleElement type="headerRow" dxfId="3"/>
-      <tableStyleElement type="firstRowStripe" dxfId="2"/>
-      <tableStyleElement type="secondRowStripe" dxfId="1"/>
+      <tableStyleElement type="wholeTable" size="0" dxfId="3"/>
+      <tableStyleElement type="headerRow" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="secondRowStripe" dxfId="0"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -1744,7 +1744,7 @@
         <v>33</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>123</v>
@@ -1772,7 +1772,7 @@
         <v>33</v>
       </c>
       <c r="C29" s="16" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>123</v>
@@ -1912,10 +1912,10 @@
         <v>140</v>
       </c>
       <c r="C34" s="3" t="s">
+        <v>156</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>141</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>142</v>
       </c>
       <c r="E34" s="3">
         <v>0.29485</v>
@@ -1924,7 +1924,7 @@
         <v>24960</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="H34" s="7"/>
       <c r="I34" s="3" t="s">
@@ -1934,13 +1934,13 @@
     </row>
     <row r="35" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>40</v>
@@ -1952,7 +1952,7 @@
         <v>9900</v>
       </c>
       <c r="G35" s="6" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="H35" s="7"/>
       <c r="I35" s="3" t="s">
@@ -1962,13 +1962,13 @@
     </row>
     <row r="36" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>38</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>40</v>
@@ -1980,7 +1980,7 @@
         <v>2105500</v>
       </c>
       <c r="G36" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="H36" s="7"/>
       <c r="I36" s="3" t="s">
@@ -1990,16 +1990,16 @@
     </row>
     <row r="37" spans="1:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="B37" s="3" t="s">
         <v>150</v>
       </c>
-      <c r="B37" s="3" t="s">
+      <c r="C37" s="3" t="s">
         <v>151</v>
       </c>
-      <c r="C37" s="3" t="s">
+      <c r="D37" s="3" t="s">
         <v>152</v>
-      </c>
-      <c r="D37" s="3" t="s">
-        <v>153</v>
       </c>
       <c r="E37">
         <v>8.6860000000000007E-2</v>
@@ -2008,7 +2008,7 @@
         <v>9620</v>
       </c>
       <c r="G37" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="H37" s="7"/>
       <c r="I37" s="3" t="s">

</xml_diff>